<commit_message>
Sin cifras de grupos ni estudiantes, sin jornada Completa y Guía solo informativa
- Modelos flexibles: la página solo dice qué modelos ofrece cada institución,
  en qué sedes y jornadas. MF ya no trae estudiantes ni repite grupos; se
  quita la pestaña de grupos de la ficha, el orden por estudiantes y los
  colores del mapa por estudiantes y grupos (queda «con modelos flexibles»).
- Jornada Completa fuera de filtros, tarjetas, fichas y datos de SINEB.
- Guía sin cifras ni botones de resultados; se eliminan «Atención e
  inclusión», «Fuentes y actualización», «Privacidad y datos de contacto» y
  «Aclaraciones y limitaciones».
- READMEs actualizados.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XfJr2rHFAKgBXnNfLfMbuH
</commit_message>
<xml_diff>
--- a/datos/instituciones_clei.xlsx
+++ b/datos/instituciones_clei.xlsx
@@ -1395,7 +1395,7 @@
     <col width="37" customWidth="1" min="7" max="7"/>
     <col width="38" customWidth="1" min="8" max="8"/>
     <col width="60" customWidth="1" min="9" max="9"/>
-    <col width="47" customWidth="1" min="10" max="10"/>
+    <col width="37" customWidth="1" min="10" max="10"/>
     <col width="15" customWidth="1" min="11" max="11"/>
     <col width="21" customWidth="1" min="12" max="12"/>
     <col width="10" customWidth="1" min="13" max="13"/>
@@ -3592,7 +3592,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Mañana, Tarde, Única, Completa</t>
+          <t>Mañana, Tarde, Única</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -6517,7 +6517,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Mañana, Tarde, Única, Completa</t>
+          <t>Mañana, Tarde, Única</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -6918,7 +6918,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>Mañana, Tarde, Única, Completa</t>
+          <t>Mañana, Tarde, Única</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -7301,7 +7301,7 @@
       </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
-          <t>Mañana, Tarde, Única, Completa, Fin de semana</t>
+          <t>Mañana, Tarde, Única, Fin de semana</t>
         </is>
       </c>
       <c r="K45" s="2" t="inlineStr">
@@ -8646,7 +8646,7 @@
       </c>
       <c r="J55" s="2" t="inlineStr">
         <is>
-          <t>Mañana, Tarde, Única, Completa, Fin de semana</t>
+          <t>Mañana, Tarde, Única, Fin de semana</t>
         </is>
       </c>
       <c r="K55" s="2" t="inlineStr">
@@ -9984,7 +9984,7 @@
       </c>
       <c r="J65" s="2" t="inlineStr">
         <is>
-          <t>Mañana, Tarde, Única, Completa, Fin de semana</t>
+          <t>Mañana, Tarde, Única, Fin de semana</t>
         </is>
       </c>
       <c r="K65" s="2" t="inlineStr">
@@ -11410,7 +11410,7 @@
       </c>
       <c r="J76" s="2" t="inlineStr">
         <is>
-          <t>Mañana, Tarde, Completa, Fin de semana</t>
+          <t>Mañana, Tarde, Fin de semana</t>
         </is>
       </c>
       <c r="K76" s="2" t="inlineStr">
@@ -11654,7 +11654,7 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>Tarde, Completa</t>
+          <t>Tarde</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -12377,7 +12377,7 @@
       </c>
       <c r="J84" s="2" t="inlineStr">
         <is>
-          <t>Mañana, Tarde, Completa, Fin de semana</t>
+          <t>Mañana, Tarde, Fin de semana</t>
         </is>
       </c>
       <c r="K84" s="2" t="inlineStr">
@@ -12733,7 +12733,7 @@
       <c r="I87" s="2" t="inlineStr"/>
       <c r="J87" s="2" t="inlineStr">
         <is>
-          <t>Mañana, Tarde, Completa, Fin de semana</t>
+          <t>Mañana, Tarde, Fin de semana</t>
         </is>
       </c>
       <c r="K87" s="2" t="inlineStr">
@@ -12975,7 +12975,7 @@
       </c>
       <c r="J89" s="2" t="inlineStr">
         <is>
-          <t>Completa, Fin de semana</t>
+          <t>Fin de semana</t>
         </is>
       </c>
       <c r="K89" s="2" t="inlineStr">
@@ -13095,11 +13095,6 @@
           <t>4485168</t>
         </is>
       </c>
-      <c r="J90" t="inlineStr">
-        <is>
-          <t>Completa</t>
-        </is>
-      </c>
       <c r="K90" t="inlineStr">
         <is>
           <t>No</t>
@@ -13216,11 +13211,6 @@
           <t>colegio@lujan.edu.co</t>
         </is>
       </c>
-      <c r="J91" t="inlineStr">
-        <is>
-          <t>Completa</t>
-        </is>
-      </c>
       <c r="K91" t="inlineStr">
         <is>
           <t>No</t>
@@ -13447,7 +13437,7 @@
       </c>
       <c r="J93" s="2" t="inlineStr">
         <is>
-          <t>Mañana, Tarde, Completa, Fin de semana</t>
+          <t>Mañana, Tarde, Fin de semana</t>
         </is>
       </c>
       <c r="K93" s="2" t="inlineStr">
@@ -13939,7 +13929,7 @@
       </c>
       <c r="J97" s="2" t="inlineStr">
         <is>
-          <t>Mañana, Tarde, Completa, Fin de semana</t>
+          <t>Mañana, Tarde, Fin de semana</t>
         </is>
       </c>
       <c r="K97" s="2" t="inlineStr">
@@ -14755,7 +14745,7 @@
       </c>
       <c r="J104" s="2" t="inlineStr">
         <is>
-          <t>Mañana, Tarde, Completa, Fin de semana</t>
+          <t>Mañana, Tarde, Fin de semana</t>
         </is>
       </c>
       <c r="K104" s="2" t="inlineStr">
@@ -15116,7 +15106,7 @@
       </c>
       <c r="J107" s="2" t="inlineStr">
         <is>
-          <t>Mañana, Tarde, Completa, Fin de semana</t>
+          <t>Mañana, Tarde, Fin de semana</t>
         </is>
       </c>
       <c r="K107" s="2" t="inlineStr">
@@ -16466,7 +16456,7 @@
     <col width="26" customWidth="1" min="6" max="6"/>
     <col width="38" customWidth="1" min="7" max="7"/>
     <col width="48" customWidth="1" min="8" max="8"/>
-    <col width="47" customWidth="1" min="9" max="9"/>
+    <col width="37" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
     <col width="21" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
@@ -18578,7 +18568,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Mañana, Tarde, Única, Completa</t>
+          <t>Mañana, Tarde, Única</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -21393,7 +21383,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Mañana, Tarde, Única, Completa</t>
+          <t>Mañana, Tarde, Única</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -21779,7 +21769,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Mañana, Tarde, Única, Completa</t>
+          <t>Mañana, Tarde, Única</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
@@ -22147,7 +22137,7 @@
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>Mañana, Tarde, Única, Completa, Fin de semana</t>
+          <t>Mañana, Tarde, Única, Fin de semana</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr">
@@ -23442,7 +23432,7 @@
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
-          <t>Mañana, Tarde, Única, Completa, Fin de semana</t>
+          <t>Mañana, Tarde, Única, Fin de semana</t>
         </is>
       </c>
       <c r="J55" s="2" t="inlineStr">
@@ -24730,7 +24720,7 @@
       </c>
       <c r="I65" s="2" t="inlineStr">
         <is>
-          <t>Mañana, Tarde, Única, Completa, Fin de semana</t>
+          <t>Mañana, Tarde, Única, Fin de semana</t>
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr">
@@ -25615,7 +25605,7 @@
     <col width="37" customWidth="1" min="4" max="4"/>
     <col width="29" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
@@ -26266,7 +26256,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Mañana, Tarde, Completa, Fin de semana</t>
+          <t>Mañana, Tarde, Fin de semana</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -26498,7 +26488,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Tarde, Completa</t>
+          <t>Tarde</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -27181,7 +27171,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Mañana, Tarde, Completa, Fin de semana</t>
+          <t>Mañana, Tarde, Fin de semana</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -27518,7 +27508,7 @@
       <c r="F17" s="2" t="inlineStr"/>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Mañana, Tarde, Completa, Fin de semana</t>
+          <t>Mañana, Tarde, Fin de semana</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -27746,7 +27736,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Completa, Fin de semana</t>
+          <t>Fin de semana</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -27861,11 +27851,6 @@
           <t>4485168</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Completa</t>
-        </is>
-      </c>
       <c r="H20" t="inlineStr">
         <is>
           <t>No</t>
@@ -27977,11 +27962,6 @@
           <t>colegio@lujan.edu.co</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>Completa</t>
-        </is>
-      </c>
       <c r="H21" t="inlineStr">
         <is>
           <t>No</t>
@@ -28196,7 +28176,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Mañana, Tarde, Completa, Fin de semana</t>
+          <t>Mañana, Tarde, Fin de semana</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -28660,7 +28640,7 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Mañana, Tarde, Completa, Fin de semana</t>
+          <t>Mañana, Tarde, Fin de semana</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -29433,7 +29413,7 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Mañana, Tarde, Completa, Fin de semana</t>
+          <t>Mañana, Tarde, Fin de semana</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -29775,7 +29755,7 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Mañana, Tarde, Completa, Fin de semana</t>
+          <t>Mañana, Tarde, Fin de semana</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -31056,7 +31036,7 @@
     <col width="60" customWidth="1" min="7" max="7"/>
     <col width="39" customWidth="1" min="8" max="8"/>
     <col width="60" customWidth="1" min="9" max="9"/>
-    <col width="47" customWidth="1" min="10" max="10"/>
+    <col width="37" customWidth="1" min="10" max="10"/>
     <col width="15" customWidth="1" min="11" max="11"/>
     <col width="21" customWidth="1" min="12" max="12"/>
     <col width="10" customWidth="1" min="13" max="13"/>
@@ -31337,11 +31317,6 @@
           <t>ce.juanandrespatino@medellin.gov.co</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Completa</t>
-        </is>
-      </c>
       <c r="K2" t="inlineStr">
         <is>
           <t>No</t>
@@ -31522,7 +31497,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Única, Completa</t>
+          <t>Única</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -31886,11 +31861,6 @@
           <t>ce.permanentemazo@medellin.gov.co</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Completa</t>
-        </is>
-      </c>
       <c r="K5" t="inlineStr">
         <is>
           <t>No</t>
@@ -37889,7 +37859,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Mañana, Tarde, Única, Completa</t>
+          <t>Mañana, Tarde, Única</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -46335,7 +46305,7 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>Mañana, Tarde, Única, Completa</t>
+          <t>Mañana, Tarde, Única</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
@@ -47639,7 +47609,7 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>Mañana, Tarde, Única, Completa</t>
+          <t>Mañana, Tarde, Única</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
@@ -48574,7 +48544,7 @@
       </c>
       <c r="J94" s="2" t="inlineStr">
         <is>
-          <t>Mañana, Tarde, Única, Completa, Fin de semana</t>
+          <t>Mañana, Tarde, Única, Fin de semana</t>
         </is>
       </c>
       <c r="K94" s="2" t="inlineStr">
@@ -55282,7 +55252,7 @@
       </c>
       <c r="J130" s="2" t="inlineStr">
         <is>
-          <t>Mañana, Tarde, Única, Completa, Fin de semana</t>
+          <t>Mañana, Tarde, Única, Fin de semana</t>
         </is>
       </c>
       <c r="K130" s="2" t="inlineStr">
@@ -55670,7 +55640,7 @@
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>Mañana, Tarde, Única, Completa</t>
+          <t>Mañana, Tarde, Única</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
@@ -59585,7 +59555,7 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>Mañana, Tarde, Única, Completa, Fin de semana</t>
+          <t>Mañana, Tarde, Única, Fin de semana</t>
         </is>
       </c>
       <c r="K153" s="2" t="inlineStr">
@@ -61844,7 +61814,7 @@
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>Mañana, Tarde, Única, Completa</t>
+          <t>Mañana, Tarde, Única</t>
         </is>
       </c>
       <c r="K165" t="inlineStr">
@@ -62198,11 +62168,6 @@
           <t>inamejia@educame.gov.co</t>
         </is>
       </c>
-      <c r="J167" t="inlineStr">
-        <is>
-          <t>Completa</t>
-        </is>
-      </c>
       <c r="K167" t="inlineStr">
         <is>
           <t>No</t>
@@ -62368,7 +62333,7 @@
       </c>
       <c r="J168" t="inlineStr">
         <is>
-          <t>Mañana, Completa</t>
+          <t>Mañana</t>
         </is>
       </c>
       <c r="K168" t="inlineStr">
@@ -63268,7 +63233,7 @@
       </c>
       <c r="J173" s="2" t="inlineStr">
         <is>
-          <t>Mañana, Tarde, Completa, Fin de semana</t>
+          <t>Mañana, Tarde, Fin de semana</t>
         </is>
       </c>
       <c r="K173" s="2" t="inlineStr">
@@ -63626,7 +63591,7 @@
       </c>
       <c r="J175" t="inlineStr">
         <is>
-          <t>Tarde, Completa</t>
+          <t>Tarde</t>
         </is>
       </c>
       <c r="K175" t="inlineStr">
@@ -64150,7 +64115,7 @@
       </c>
       <c r="J178" t="inlineStr">
         <is>
-          <t>Mañana, Tarde, Completa</t>
+          <t>Mañana, Tarde</t>
         </is>
       </c>
       <c r="K178" t="inlineStr">
@@ -65037,7 +65002,7 @@
       </c>
       <c r="J183" s="2" t="inlineStr">
         <is>
-          <t>Mañana, Tarde, Completa, Fin de semana</t>
+          <t>Mañana, Tarde, Fin de semana</t>
         </is>
       </c>
       <c r="K183" s="2" t="inlineStr">
@@ -65401,7 +65366,7 @@
       <c r="I185" s="2" t="inlineStr"/>
       <c r="J185" s="2" t="inlineStr">
         <is>
-          <t>Mañana, Tarde, Completa, Fin de semana</t>
+          <t>Mañana, Tarde, Fin de semana</t>
         </is>
       </c>
       <c r="K185" s="2" t="inlineStr">
@@ -65757,7 +65722,7 @@
       </c>
       <c r="J187" s="2" t="inlineStr">
         <is>
-          <t>Completa, Fin de semana</t>
+          <t>Fin de semana</t>
         </is>
       </c>
       <c r="K187" s="2" t="inlineStr">
@@ -65934,11 +65899,6 @@
           <t>4485168</t>
         </is>
       </c>
-      <c r="J188" t="inlineStr">
-        <is>
-          <t>Completa</t>
-        </is>
-      </c>
       <c r="K188" t="inlineStr">
         <is>
           <t>No</t>
@@ -66117,11 +66077,6 @@
           <t>colegio@lujan.edu.co</t>
         </is>
       </c>
-      <c r="J189" t="inlineStr">
-        <is>
-          <t>Completa</t>
-        </is>
-      </c>
       <c r="K189" t="inlineStr">
         <is>
           <t>No</t>
@@ -66472,7 +66427,7 @@
       </c>
       <c r="J191" s="2" t="inlineStr">
         <is>
-          <t>Mañana, Tarde, Completa, Fin de semana</t>
+          <t>Mañana, Tarde, Fin de semana</t>
         </is>
       </c>
       <c r="K191" s="2" t="inlineStr">
@@ -68076,7 +68031,7 @@
       </c>
       <c r="J200" s="2" t="inlineStr">
         <is>
-          <t>Mañana, Tarde, Completa, Fin de semana</t>
+          <t>Mañana, Tarde, Fin de semana</t>
         </is>
       </c>
       <c r="K200" s="2" t="inlineStr">
@@ -68613,7 +68568,7 @@
       </c>
       <c r="J203" s="2" t="inlineStr">
         <is>
-          <t>Mañana, Tarde, Completa, Fin de semana</t>
+          <t>Mañana, Tarde, Fin de semana</t>
         </is>
       </c>
       <c r="K203" s="2" t="inlineStr">

</xml_diff>